<commit_message>
Replace catalog beads with new_input SKUs and refresh Shopify CSV.
Keep accessories unchanged, remap plaza bead formulas to the new catalog, and ship product images for GitHub Pages.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/plaza_designs.xlsx
+++ b/data/plaza_designs.xlsx
@@ -399,26 +399,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:R8"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="15.83203125" customWidth="1"/>
-    <col min="4" max="4" width="13.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="15.83203125" customWidth="1"/>
-    <col min="7" max="7" width="12.83203125" customWidth="1"/>
-    <col min="8" max="8" width="12.83203125" customWidth="1"/>
-    <col min="9" max="9" width="12.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="12.83203125" customWidth="1"/>
-    <col min="12" max="12" width="18.83203125" customWidth="1"/>
-    <col min="13" max="13" width="14.83203125" customWidth="1"/>
-    <col min="14" max="14" width="12.83203125" customWidth="1"/>
-    <col min="15" max="15" width="12.83203125" customWidth="1"/>
-    <col min="16" max="16" width="13.83203125" customWidth="1"/>
-    <col min="17" max="17" width="13.83203125" customWidth="1"/>
-    <col min="18" max="18" width="12.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -511,7 +491,7 @@
         <v>/plaza/pub-e08d746d-a3c1-4af2-b999-affff7c64ac5.png</v>
       </c>
       <c r="L2" t="str">
-        <v>jsxh_spc_5|nbj_cysl_6|jhy_stn_6|nbj_cysl_6|jsxh_spc_5|nbj_cysl_6|jhy_stn_6|jsxh_spc_5|nbj_cysl_6|jhy_stn_6|jsxh_spc_5|nbj_cysl_6|jhy_stn_6|jsxh_spc_5|nbj_cysl_6|jhy_stn_6|jsxh_spc_5|nbj_cysl_6|jhy_stn_6|jsxh_spc_5|nbj_cysl_6|jhy_stn_6</v>
+        <v>jsxh_spc_5|bsj_cysl_6|hyes_stn_6|bsj_cysl_6|jsxh_spc_5|bsj_cysl_6|hyes_stn_6|jsxh_spc_5|bsj_cysl_6|hyes_stn_6|jsxh_spc_5|bsj_cysl_6|hyes_stn_6|jsxh_spc_5|bsj_cysl_6|hyes_stn_6|jsxh_spc_5|bsj_cysl_6|hyes_stn_6|jsxh_spc_5|bsj_cysl_6|hyes_stn_6</v>
       </c>
       <c r="M2" t="str">
         <v>2026-07-22T07:19:34.452Z</v>
@@ -567,7 +547,7 @@
         <v>/plaza/pub-dca45881-9c67-4dd0-b6f7-c1fcfbe3bcf4.png</v>
       </c>
       <c r="L3" t="str">
-        <v>lfj_cysl_6|kqs_stn_6|lys_stn_6|lpts_stn_6|syyl_pnd_2|lfj_cysl_6|kqs_stn_6|lys_stn_6|lpts_stn_6|jd_pnd_2|lfj_cysl_6|kqs_stn_6|lys_stn_6|lpts_stn_6|bmw_pnd_2|lfj_cysl_6|lys_stn_6|kqs_stn_6|lpts_stn_6|gsxx_pnd_2|lfj_cysl_6|lys_stn_6|kqs_stn_6|cyhdls_pnd_2|lpts_stn_6</v>
+        <v>lfj_cysl_8|kqs_stn_6|lys_stn_6|pts_stn_6|syyl_pnd_2|lfj_cysl_8|kqs_stn_6|lys_stn_6|pts_stn_6|jd_pnd_2|lfj_cysl_8|kqs_stn_6|lys_stn_6|pts_stn_6|bmw_pnd_2|lfj_cysl_8|lys_stn_6|kqs_stn_6|pts_stn_6|gsxx_pnd_2|lfj_cysl_8|lys_stn_6|kqs_stn_6|cyhdls_pnd_2|pts_stn_6</v>
       </c>
       <c r="M3" t="str">
         <v>2026-07-22T07:18:20.424Z</v>
@@ -608,7 +588,7 @@
         <v>59</v>
       </c>
       <c r="G4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H4" t="str">
         <v>published</v>
@@ -629,7 +609,7 @@
         <v>2026-07-22T07:11:05.918Z</v>
       </c>
       <c r="N4" t="str">
-        <v>2026-07-22T07:11:05.934Z</v>
+        <v>2026-07-26T06:25:14.610Z</v>
       </c>
       <c r="O4">
         <v>0</v>
@@ -679,7 +659,7 @@
         <v>/plaza/pub-283e7097-b146-47db-82be-84a7b0ab7d3e.png</v>
       </c>
       <c r="L5" t="str">
-        <v>nbj_cysl_6|nbj_cysl_6|nbj_cysl_6|nyl_stn_6|nyl_stn_6|nyl_stn_6|lpts_stn_6|lpts_stn_6|lpts_stn_6|hsj_cysl_6|hsj_cysl_6|hsj_cysl_6|lys_stn_6|lys_stn_6|lys_stn_6|xyczsj_cysl_6|xyczsj_cysl_6|xyczsj_cysl_6|ccs_stn_6|ccs_stn_6|ccs_stn_6|ljs_stn_6|ljs_stn_6|ljs_stn_6</v>
+        <v>bsj_cysl_6|bsj_cysl_6|bsj_cysl_6|hlb_stn_6|hlb_stn_6|hlb_stn_6|pts_stn_6|pts_stn_6|pts_stn_6|hsj_cysl_6|hsj_cysl_6|hsj_cysl_6|lys_stn_6|lys_stn_6|lys_stn_6|zsj_cysl_6|zsj_cysl_6|zsj_cysl_6|tys_stn_6|tys_stn_6|tys_stn_6|ljs_stn_6|ljs_stn_6|ljs_stn_6</v>
       </c>
       <c r="M5" t="str">
         <v>2026-07-22T07:10:43.463Z</v>
@@ -720,7 +700,7 @@
         <v>39</v>
       </c>
       <c r="G6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H6" t="str">
         <v>published</v>
@@ -735,13 +715,13 @@
         <v>/plaza/pub-bf77b5cd-cf3b-489e-9e91-e777c28c1d4c.png</v>
       </c>
       <c r="L6" t="str">
-        <v>cysy_spc_6|dszz_prl_8|cysy_spc_6|dszz_prl_8|cysy_spc_6|dszz_prl_8|cysy_spc_6|dszz_prl_8|cysy_spc_6|dszz_prl_8|cysy_spc_6|dszz_prl_8|cysy_spc_6|dszz_prl_8|cysy_spc_6|dszz_prl_8|cysy_spc_6|dszz_prl_8|cysy_spc_6|dszz_prl_8</v>
+        <v>cysy_spc_6|dszzhu_prl_8|cysy_spc_6|dszzhu_prl_8|cysy_spc_6|dszzhu_prl_8|cysy_spc_6|dszzhu_prl_8|cysy_spc_6|dszzhu_prl_8|cysy_spc_6|dszzhu_prl_8|cysy_spc_6|dszzhu_prl_8|cysy_spc_6|dszzhu_prl_8|cysy_spc_6|dszzhu_prl_8|cysy_spc_6|dszzhu_prl_8</v>
       </c>
       <c r="M6" t="str">
         <v>2026-07-22T07:10:15.766Z</v>
       </c>
       <c r="N6" t="str">
-        <v>2026-07-22T07:10:15.778Z</v>
+        <v>2026-07-23T18:02:27.019Z</v>
       </c>
       <c r="O6">
         <v>0</v>
@@ -791,7 +771,7 @@
         <v>/plaza/pub-029d61e7-facb-4963-9d7b-440fe70b8343.png</v>
       </c>
       <c r="L7" t="str">
-        <v>dszz_prl_8|dszz_prl_8|dszz_prl_8|dszz_prl_8|dszz_prl_8|dszz_prl_6|dszz_prl_6|dszz_prl_6|dszz_prl_6|dszz_prl_6|dszz_prl_6|dszz_prl_6|dszz_prl_8|dszz_prl_8|dszz_prl_8|dszz_prl_10|dszz_prl_10|dszz_prl_10|dszz_prl_10|dszz_prl_10|dszz_prl_10|dszz_prl_10</v>
+        <v>dszzhu_prl_8|dszzhu_prl_8|dszzhu_prl_8|dszzhu_prl_8|dszzhu_prl_8|dszzhu_prl_6|dszzhu_prl_6|dszzhu_prl_6|dszzhu_prl_6|dszzhu_prl_6|dszzhu_prl_6|dszzhu_prl_6|dszzhu_prl_8|dszzhu_prl_8|dszzhu_prl_8|dszzhu_prl_10|dszzhu_prl_10|dszzhu_prl_10|dszzhu_prl_10|dszzhu_prl_10|dszzhu_prl_10|dszzhu_prl_10</v>
       </c>
       <c r="M7" t="str">
         <v>2026-07-22T07:09:21.985Z</v>
@@ -878,12 +858,6 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D19"/>
-  <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" customWidth="1"/>
-    <col min="3" max="3" width="10.83203125" customWidth="1"/>
-    <col min="4" max="4" width="64.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">

</xml_diff>

<commit_message>
Reopen plaza publish and clear all existing plaza designs.
Remove the completed-order gate on publish, wipe UGC/master plaza data after the catalog swap, and bump localStorage keys so clients drop stale publishes.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/plaza_designs.xlsx
+++ b/data/plaza_designs.xlsx
@@ -398,7 +398,27 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R8"/>
+  <dimension ref="A1:R1"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="15.83203125" customWidth="1"/>
+    <col min="4" max="4" width="13.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="15.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+    <col min="8" max="8" width="12.83203125" customWidth="1"/>
+    <col min="9" max="9" width="12.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="12.83203125" customWidth="1"/>
+    <col min="12" max="12" width="18.83203125" customWidth="1"/>
+    <col min="13" max="13" width="14.83203125" customWidth="1"/>
+    <col min="14" max="14" width="12.83203125" customWidth="1"/>
+    <col min="15" max="15" width="12.83203125" customWidth="1"/>
+    <col min="16" max="16" width="13.83203125" customWidth="1"/>
+    <col min="17" max="17" width="13.83203125" customWidth="1"/>
+    <col min="18" max="18" width="12.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -456,401 +476,9 @@
         <v>notes</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>pub-e08d746d-a3c1-4af2-b999-affff7c64ac5</v>
-      </c>
-      <c r="B2" t="str">
-        <v>金色琉璃</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Linda</v>
-      </c>
-      <c r="D2" t="str">
-        <v>912525</v>
-      </c>
-      <c r="E2" t="str">
-        <v>靈珠護佑😄平安常伴</v>
-      </c>
-      <c r="F2">
-        <v>89</v>
-      </c>
-      <c r="G2">
-        <v>0</v>
-      </c>
-      <c r="H2" t="str">
-        <v>published</v>
-      </c>
-      <c r="I2" t="str">
-        <v>user</v>
-      </c>
-      <c r="J2" t="str">
-        <v>db41a9f0-73b7-410a-9b85-d3e2ddc63e38</v>
-      </c>
-      <c r="K2" t="str">
-        <v>/plaza/pub-e08d746d-a3c1-4af2-b999-affff7c64ac5.png</v>
-      </c>
-      <c r="L2" t="str">
-        <v>jsxh_spc_5|bsj_cysl_6|hyes_stn_6|bsj_cysl_6|jsxh_spc_5|bsj_cysl_6|hyes_stn_6|jsxh_spc_5|bsj_cysl_6|hyes_stn_6|jsxh_spc_5|bsj_cysl_6|hyes_stn_6|jsxh_spc_5|bsj_cysl_6|hyes_stn_6|jsxh_spc_5|bsj_cysl_6|hyes_stn_6|jsxh_spc_5|bsj_cysl_6|hyes_stn_6</v>
-      </c>
-      <c r="M2" t="str">
-        <v>2026-07-22T07:19:34.452Z</v>
-      </c>
-      <c r="N2" t="str">
-        <v>2026-07-22T07:55:04.878Z</v>
-      </c>
-      <c r="O2">
-        <v>0</v>
-      </c>
-      <c r="P2">
-        <v>0</v>
-      </c>
-      <c r="Q2">
-        <v>0</v>
-      </c>
-      <c r="R2" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>pub-dca45881-9c67-4dd0-b6f7-c1fcfbe3bcf4</v>
-      </c>
-      <c r="B3" t="str">
-        <v>捕夢網</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Mia</v>
-      </c>
-      <c r="D3" t="str">
-        <v>912525</v>
-      </c>
-      <c r="E3" t="str">
-        <v>青嵐 · 攬夢 · 捕夢</v>
-      </c>
-      <c r="F3">
-        <v>99</v>
-      </c>
-      <c r="G3">
-        <v>0</v>
-      </c>
-      <c r="H3" t="str">
-        <v>published</v>
-      </c>
-      <c r="I3" t="str">
-        <v>user</v>
-      </c>
-      <c r="J3" t="str">
-        <v>5b78023d-6695-4ce9-800d-d422d37b9b45</v>
-      </c>
-      <c r="K3" t="str">
-        <v>/plaza/pub-dca45881-9c67-4dd0-b6f7-c1fcfbe3bcf4.png</v>
-      </c>
-      <c r="L3" t="str">
-        <v>lfj_cysl_8|kqs_stn_6|lys_stn_6|pts_stn_6|syyl_pnd_2|lfj_cysl_8|kqs_stn_6|lys_stn_6|pts_stn_6|jd_pnd_2|lfj_cysl_8|kqs_stn_6|lys_stn_6|pts_stn_6|bmw_pnd_2|lfj_cysl_8|lys_stn_6|kqs_stn_6|pts_stn_6|gsxx_pnd_2|lfj_cysl_8|lys_stn_6|kqs_stn_6|cyhdls_pnd_2|pts_stn_6</v>
-      </c>
-      <c r="M3" t="str">
-        <v>2026-07-22T07:18:20.424Z</v>
-      </c>
-      <c r="N3" t="str">
-        <v>2026-07-22T07:55:02.021Z</v>
-      </c>
-      <c r="O3">
-        <v>0</v>
-      </c>
-      <c r="P3">
-        <v>0</v>
-      </c>
-      <c r="Q3">
-        <v>0</v>
-      </c>
-      <c r="R3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>pub-a81f6111-a00b-4f28-8b16-8eb95c21fd44</v>
-      </c>
-      <c r="B4" t="str">
-        <v>金玉滿堂</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Linda</v>
-      </c>
-      <c r="D4" t="str">
-        <v>912525</v>
-      </c>
-      <c r="E4" t="str">
-        <v>送媽媽的禮物</v>
-      </c>
-      <c r="F4">
-        <v>59</v>
-      </c>
-      <c r="G4">
-        <v>1</v>
-      </c>
-      <c r="H4" t="str">
-        <v>published</v>
-      </c>
-      <c r="I4" t="str">
-        <v>user</v>
-      </c>
-      <c r="J4" t="str">
-        <v>a52f6eb7-fc15-4c99-9e9d-4439d0bdd750</v>
-      </c>
-      <c r="K4" t="str">
-        <v>/plaza/pub-a81f6111-a00b-4f28-8b16-8eb95c21fd44.png</v>
-      </c>
-      <c r="L4" t="str">
-        <v>jslzzy_spc_8|hmn_agt_6|jsxz_spc_6|hmn_agt_6|jsxz_spc_6|hmn_agt_6|jsxz_spc_6|hmn_agt_6|jsxz_spc_6|lkjf_pnd_2|hmn_agt_6|jsxz_spc_6|hmn_agt_6|jsxz_spc_6|hmn_agt_6|jsxz_spc_6|hmn_agt_6|jsxz_spc_6|hmn_agt_6|jsxz_spc_6|hmn_agt_6|jsxz_spc_6|hmn_agt_6</v>
-      </c>
-      <c r="M4" t="str">
-        <v>2026-07-22T07:11:05.918Z</v>
-      </c>
-      <c r="N4" t="str">
-        <v>2026-07-26T06:25:14.610Z</v>
-      </c>
-      <c r="O4">
-        <v>0</v>
-      </c>
-      <c r="P4">
-        <v>0</v>
-      </c>
-      <c r="Q4">
-        <v>0</v>
-      </c>
-      <c r="R4" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>pub-283e7097-b146-47db-82be-84a7b0ab7d3e</v>
-      </c>
-      <c r="B5" t="str">
-        <v>彩虹</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Linda</v>
-      </c>
-      <c r="D5" t="str">
-        <v>912525</v>
-      </c>
-      <c r="E5" t="str">
-        <v>來一首周杰倫的彩虹～</v>
-      </c>
-      <c r="F5">
-        <v>39</v>
-      </c>
-      <c r="G5">
-        <v>1</v>
-      </c>
-      <c r="H5" t="str">
-        <v>published</v>
-      </c>
-      <c r="I5" t="str">
-        <v>user</v>
-      </c>
-      <c r="J5" t="str">
-        <v>af8d40c1-52a9-4f02-a09e-d9effe780820</v>
-      </c>
-      <c r="K5" t="str">
-        <v>/plaza/pub-283e7097-b146-47db-82be-84a7b0ab7d3e.png</v>
-      </c>
-      <c r="L5" t="str">
-        <v>bsj_cysl_6|bsj_cysl_6|bsj_cysl_6|hlb_stn_6|hlb_stn_6|hlb_stn_6|pts_stn_6|pts_stn_6|pts_stn_6|hsj_cysl_6|hsj_cysl_6|hsj_cysl_6|lys_stn_6|lys_stn_6|lys_stn_6|zsj_cysl_6|zsj_cysl_6|zsj_cysl_6|tys_stn_6|tys_stn_6|tys_stn_6|ljs_stn_6|ljs_stn_6|ljs_stn_6</v>
-      </c>
-      <c r="M5" t="str">
-        <v>2026-07-22T07:10:43.463Z</v>
-      </c>
-      <c r="N5" t="str">
-        <v>2026-07-22T13:33:55.782Z</v>
-      </c>
-      <c r="O5">
-        <v>0</v>
-      </c>
-      <c r="P5">
-        <v>0</v>
-      </c>
-      <c r="Q5">
-        <v>0</v>
-      </c>
-      <c r="R5" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>pub-bf77b5cd-cf3b-489e-9e91-e777c28c1d4c</v>
-      </c>
-      <c r="B6" t="str">
-        <v>珍珠項鍊</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Mia</v>
-      </c>
-      <c r="D6" t="str">
-        <v>912525</v>
-      </c>
-      <c r="E6" t="str">
-        <v/>
-      </c>
-      <c r="F6">
-        <v>39</v>
-      </c>
-      <c r="G6">
-        <v>1</v>
-      </c>
-      <c r="H6" t="str">
-        <v>published</v>
-      </c>
-      <c r="I6" t="str">
-        <v>user</v>
-      </c>
-      <c r="J6" t="str">
-        <v>932607f9-30dd-4088-b79a-8bee4688bf98</v>
-      </c>
-      <c r="K6" t="str">
-        <v>/plaza/pub-bf77b5cd-cf3b-489e-9e91-e777c28c1d4c.png</v>
-      </c>
-      <c r="L6" t="str">
-        <v>cysy_spc_6|dszzhu_prl_8|cysy_spc_6|dszzhu_prl_8|cysy_spc_6|dszzhu_prl_8|cysy_spc_6|dszzhu_prl_8|cysy_spc_6|dszzhu_prl_8|cysy_spc_6|dszzhu_prl_8|cysy_spc_6|dszzhu_prl_8|cysy_spc_6|dszzhu_prl_8|cysy_spc_6|dszzhu_prl_8|cysy_spc_6|dszzhu_prl_8</v>
-      </c>
-      <c r="M6" t="str">
-        <v>2026-07-22T07:10:15.766Z</v>
-      </c>
-      <c r="N6" t="str">
-        <v>2026-07-23T18:02:27.019Z</v>
-      </c>
-      <c r="O6">
-        <v>0</v>
-      </c>
-      <c r="P6">
-        <v>0</v>
-      </c>
-      <c r="Q6">
-        <v>0</v>
-      </c>
-      <c r="R6" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>pub-029d61e7-facb-4963-9d7b-440fe70b8343</v>
-      </c>
-      <c r="B7" t="str">
-        <v>漸變</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Mia</v>
-      </c>
-      <c r="D7" t="str">
-        <v>912525</v>
-      </c>
-      <c r="E7" t="str">
-        <v>小眾珍珠漸變手串</v>
-      </c>
-      <c r="F7">
-        <v>19</v>
-      </c>
-      <c r="G7">
-        <v>1</v>
-      </c>
-      <c r="H7" t="str">
-        <v>published</v>
-      </c>
-      <c r="I7" t="str">
-        <v>user</v>
-      </c>
-      <c r="J7" t="str">
-        <v>690a6253-00e8-4183-b004-a25e5c2fe10e</v>
-      </c>
-      <c r="K7" t="str">
-        <v>/plaza/pub-029d61e7-facb-4963-9d7b-440fe70b8343.png</v>
-      </c>
-      <c r="L7" t="str">
-        <v>dszzhu_prl_8|dszzhu_prl_8|dszzhu_prl_8|dszzhu_prl_8|dszzhu_prl_8|dszzhu_prl_6|dszzhu_prl_6|dszzhu_prl_6|dszzhu_prl_6|dszzhu_prl_6|dszzhu_prl_6|dszzhu_prl_6|dszzhu_prl_8|dszzhu_prl_8|dszzhu_prl_8|dszzhu_prl_10|dszzhu_prl_10|dszzhu_prl_10|dszzhu_prl_10|dszzhu_prl_10|dszzhu_prl_10|dszzhu_prl_10</v>
-      </c>
-      <c r="M7" t="str">
-        <v>2026-07-22T07:09:21.985Z</v>
-      </c>
-      <c r="N7" t="str">
-        <v>2026-07-23T09:17:30.695Z</v>
-      </c>
-      <c r="O7">
-        <v>0</v>
-      </c>
-      <c r="P7">
-        <v>0</v>
-      </c>
-      <c r="Q7">
-        <v>0</v>
-      </c>
-      <c r="R7" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>pub-dd0a48cc-474f-4cfe-99bf-33b84fa8558d</v>
-      </c>
-      <c r="B8" t="str">
-        <v>海洋之淚</v>
-      </c>
-      <c r="C8" t="str">
-        <v>L</v>
-      </c>
-      <c r="D8" t="str">
-        <v>912525</v>
-      </c>
-      <c r="E8" t="str">
-        <v>海洋之淚，凝萃幽藍</v>
-      </c>
-      <c r="F8">
-        <v>99</v>
-      </c>
-      <c r="G8">
-        <v>0</v>
-      </c>
-      <c r="H8" t="str">
-        <v>published</v>
-      </c>
-      <c r="I8" t="str">
-        <v>user</v>
-      </c>
-      <c r="J8" t="str">
-        <v>6ee6477a-6c49-4bb1-ab0e-b38a63ba1644</v>
-      </c>
-      <c r="K8" t="str">
-        <v>/plaza/pub-dd0a48cc-474f-4cfe-99bf-33b84fa8558d.png</v>
-      </c>
-      <c r="L8" t="str">
-        <v>qjs_stn_8|xgszs_spc_5|qjs_stn_8|xgszs_spc_5|qjs_stn_8|xgszs_spc_5|qjs_stn_8|xgszs_spc_5|syc_pnd_2|xgszs_spc_5|qjs_stn_8|xgszs_spc_5|qjs_stn_8|xgszs_spc_5|qjs_stn_8|xgszs_spc_5|qjs_stn_8|xgszs_spc_5|qjs_stn_8|xgszs_spc_5|qjs_stn_8|xgszs_spc_5</v>
-      </c>
-      <c r="M8" t="str">
-        <v>2026-07-22T07:08:36.527Z</v>
-      </c>
-      <c r="N8" t="str">
-        <v>2026-07-22T07:08:36.541Z</v>
-      </c>
-      <c r="O8">
-        <v>0</v>
-      </c>
-      <c r="P8">
-        <v>0</v>
-      </c>
-      <c r="Q8">
-        <v>0</v>
-      </c>
-      <c r="R8" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:R8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:R1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -858,6 +486,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D19"/>
+  <cols>
+    <col min="1" max="1" width="20.83203125" customWidth="1"/>
+    <col min="2" max="2" width="10.83203125" customWidth="1"/>
+    <col min="3" max="3" width="10.83203125" customWidth="1"/>
+    <col min="4" max="4" width="64.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">

</xml_diff>